<commit_message>
changed two very small refund funds to be excluded in gap analysis. Totals do not change.
</commit_message>
<xml_diff>
--- a/inputs/funds_ab_in.xlsx
+++ b/inputs/funds_ab_in.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aleaw\Documents\PhD Fall 2021 - Spring 2022\Merriman RA\Fiscal Futures IGPA\Fiscal-Future-Topics\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E824081-D7C9-4948-8DFD-8791C7688F25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B53BEA-9251-4FD8-83E6-4CC59B2410B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10335" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -136,7 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9865" uniqueCount="2663">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9866" uniqueCount="2663">
   <si>
     <t>fund</t>
   </si>
@@ -8284,7 +8284,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -8336,6 +8336,8 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8483,7 +8485,7 @@
       <sheetName val="Sheet1"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
+      <sheetData sheetId="0" refreshError="1"/>
       <sheetData sheetId="1"/>
     </sheetDataSet>
   </externalBook>
@@ -39891,7 +39893,7 @@
       <c r="G115" s="28">
         <v>1</v>
       </c>
-      <c r="H115" s="1" t="s">
+      <c r="H115" s="2" t="s">
         <v>2356</v>
       </c>
       <c r="I115" s="1" t="s">
@@ -44937,7 +44939,7 @@
       <c r="G268" s="28">
         <v>1</v>
       </c>
-      <c r="H268" s="1" t="s">
+      <c r="H268" s="2" t="s">
         <v>2356</v>
       </c>
       <c r="I268" s="1" t="s">
@@ -48202,10 +48204,10 @@
       <c r="G367" s="28">
         <v>1</v>
       </c>
-      <c r="H367" s="18" t="s">
-        <v>2306</v>
-      </c>
-      <c r="I367" s="18" t="s">
+      <c r="H367" s="37" t="s">
+        <v>2356</v>
+      </c>
+      <c r="I367" s="38" t="s">
         <v>1594</v>
       </c>
       <c r="J367" s="1" t="s">
@@ -48235,10 +48237,10 @@
       <c r="G368" s="28">
         <v>1</v>
       </c>
-      <c r="H368" s="1">
-        <v>0</v>
-      </c>
-      <c r="I368" s="1" t="s">
+      <c r="H368" s="38">
+        <v>0</v>
+      </c>
+      <c r="I368" s="38" t="s">
         <v>1595</v>
       </c>
       <c r="J368" s="1" t="s">
@@ -48268,10 +48270,10 @@
       <c r="G369" s="28">
         <v>1</v>
       </c>
-      <c r="H369" s="18" t="s">
-        <v>2306</v>
-      </c>
-      <c r="I369" s="18" t="s">
+      <c r="H369" s="37" t="s">
+        <v>2356</v>
+      </c>
+      <c r="I369" s="38" t="s">
         <v>1596</v>
       </c>
       <c r="J369" s="1" t="s">
@@ -57729,8 +57731,8 @@
       <c r="G656" s="28">
         <v>0</v>
       </c>
-      <c r="H656" s="1">
-        <v>0</v>
+      <c r="H656" s="2" t="s">
+        <v>2356</v>
       </c>
       <c r="I656" s="1" t="s">
         <v>1876</v>
@@ -66796,7 +66798,7 @@
       <c r="G931" s="28">
         <v>0</v>
       </c>
-      <c r="H931" s="1" t="s">
+      <c r="H931" s="2" t="s">
         <v>2356</v>
       </c>
       <c r="I931" s="7" t="s">

</xml_diff>